<commit_message>
Changed pre-render 	modified:   .gitignore 	modified:   .quarto/preview/lock 	modified:   _pre-render.r 	modified:   _quarto.yml 	deleted:    code/directory.rds 	modified:   documents/CCPRO_Membership_Database.xlsx 	modified:   pages/membership-directory.qmd
</commit_message>
<xml_diff>
--- a/documents/CCPRO_Membership_Database.xlsx
+++ b/documents/CCPRO_Membership_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hcc365-my.sharepoint.com/personal/rking3387_haywood_edu/Documents/LK-Obsidian/1_Projects/3_Non-Data Projects/CCPRO-Website/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{2365E0E2-A4E4-410D-B773-CA0E0058FBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{708B578E-57AD-4140-974E-1DDDC88D5240}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{2365E0E2-A4E4-410D-B773-CA0E0058FBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CEBE380-80EE-4B1C-9794-EE64B8530724}"/>
   <bookViews>
-    <workbookView xWindow="21480" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{AB234C9B-704F-466F-A7C7-F848F51275B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{AB234C9B-704F-466F-A7C7-F848F51275B9}"/>
   </bookViews>
   <sheets>
     <sheet name="New Membership" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1500" uniqueCount="777">
   <si>
     <t>current_member_name</t>
   </si>
@@ -1632,16 +1632,7 @@
     <t>hunter.ashworth@piedmontcc.edu</t>
   </si>
   <si>
-    <t>Michele Mathis</t>
-  </si>
-  <si>
     <t>Director, Research and Institutional Effectiveness</t>
-  </si>
-  <si>
-    <t>336-322-2237</t>
-  </si>
-  <si>
-    <t>Michele.Mathis@piedmontcc.edu</t>
   </si>
   <si>
     <t>Dr. Brandy Leder</t>
@@ -2746,8 +2737,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}" name="Table1" displayName="Table1" ref="A1:I185" totalsRowShown="0" dataDxfId="9">
-  <autoFilter ref="A1:I185" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}" name="Table1" displayName="Table1" ref="A1:I184" totalsRowShown="0" dataDxfId="9">
+  <autoFilter ref="A1:I184" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{3F4788B0-7800-4F61-A6A0-0A5282B58274}" name="current_member_name" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{7F07D569-61A9-4190-B534-F0A0ED69069B}" name="title" dataDxfId="7"/>
@@ -2764,8 +2755,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}" name="Table2" displayName="Table2" ref="A1:J2" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
-  <autoFilter ref="A1:J2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}" name="Table2" displayName="Table2" ref="A1:J3" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
+  <autoFilter ref="A1:J3" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1958840C-24FF-4B93-989A-E3D4C45B1A63}" name="current_member_name"/>
     <tableColumn id="2" xr3:uid="{901C16ED-C9F3-4383-BD31-77D387CB8D82}" name="updated_name"/>
@@ -3099,7 +3090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4617D616-0D58-46B6-AC53-2FFE73FE93B0}">
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -6740,25 +6731,25 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="E126" s="1" t="s">
-        <v>533</v>
+        <v>534</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>535</v>
       </c>
       <c r="F126" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H126" s="1" t="s">
         <v>15</v>
@@ -6769,28 +6760,28 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>537</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>538</v>
+        <v>534</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>539</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I127" s="6">
         <v>46118.568367997686</v>
@@ -6798,28 +6789,28 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I128" s="6">
         <v>46118.568367997686</v>
@@ -6827,22 +6818,22 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="G129" s="1" t="s">
         <v>15</v>
@@ -6856,25 +6847,25 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>549</v>
+        <v>104</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H130" s="1" t="s">
         <v>15</v>
@@ -6885,22 +6876,22 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>104</v>
+        <v>554</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="G131" s="1" t="s">
         <v>20</v>
@@ -6914,25 +6905,25 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>559</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H132" s="1" t="s">
         <v>15</v>
@@ -6946,19 +6937,19 @@
         <v>560</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>561</v>
+        <v>359</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G133" s="1" t="s">
         <v>15</v>
@@ -6972,22 +6963,22 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>359</v>
+        <v>565</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G134" s="1" t="s">
         <v>15</v>
@@ -7001,22 +6992,22 @@
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="G135" s="1" t="s">
         <v>15</v>
@@ -7030,25 +7021,25 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>564</v>
+        <v>574</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H136" s="1" t="s">
         <v>15</v>
@@ -7059,25 +7050,25 @@
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="G137" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H137" s="1" t="s">
         <v>15</v>
@@ -7088,25 +7079,25 @@
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>584</v>
       </c>
       <c r="G138" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H138" s="1" t="s">
         <v>15</v>
@@ -7126,16 +7117,16 @@
         <v>11</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="F139" s="1" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G139" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H139" s="1" t="s">
         <v>15</v>
@@ -7146,22 +7137,22 @@
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F140" s="1" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="G140" s="1" t="s">
         <v>15</v>
@@ -7175,28 +7166,28 @@
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F141" s="1" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="G141" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H141" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I141" s="6">
         <v>46118.568367997686</v>
@@ -7204,28 +7195,28 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="F142" s="1" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="G142" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H142" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I142" s="6">
         <v>46118.568367997686</v>
@@ -7233,25 +7224,25 @@
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E143" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F143" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G143" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H143" s="1" t="s">
         <v>15</v>
@@ -7262,25 +7253,25 @@
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F144" s="1" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G144" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H144" s="1" t="s">
         <v>15</v>
@@ -7291,22 +7282,22 @@
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G145" s="1" t="s">
         <v>15</v>
@@ -7320,22 +7311,22 @@
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F146" s="1" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G146" s="1" t="s">
         <v>15</v>
@@ -7349,22 +7340,22 @@
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>603</v>
+        <v>621</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="G147" s="1" t="s">
         <v>15</v>
@@ -7378,22 +7369,22 @@
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G148" s="1" t="s">
         <v>15</v>
@@ -7407,22 +7398,22 @@
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G149" s="1" t="s">
         <v>15</v>
@@ -7436,25 +7427,25 @@
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>624</v>
+        <v>634</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="G150" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H150" s="1" t="s">
         <v>15</v>
@@ -7465,25 +7456,25 @@
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="G151" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H151" s="1" t="s">
         <v>15</v>
@@ -7494,16 +7485,16 @@
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>641</v>
+        <v>171</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="E152" s="1" t="s">
         <v>642</v>
@@ -7526,19 +7517,19 @@
         <v>644</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>171</v>
+        <v>645</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>637</v>
+        <v>646</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="G153" s="1" t="s">
         <v>15</v>
@@ -7552,25 +7543,25 @@
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G154" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H154" s="1" t="s">
         <v>15</v>
@@ -7581,25 +7572,25 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="F155" s="1" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="G155" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H155" s="1" t="s">
         <v>15</v>
@@ -7610,22 +7601,22 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="G156" s="1" t="s">
         <v>15</v>
@@ -7639,16 +7630,16 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>661</v>
+        <v>36</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="E157" s="1" t="s">
         <v>663</v>
@@ -7657,7 +7648,7 @@
         <v>664</v>
       </c>
       <c r="G157" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H157" s="1" t="s">
         <v>15</v>
@@ -7671,22 +7662,22 @@
         <v>665</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>36</v>
+        <v>666</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="F158" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="G158" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H158" s="1" t="s">
         <v>15</v>
@@ -7697,16 +7688,16 @@
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>669</v>
+        <v>359</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="E159" s="1" t="s">
         <v>671</v>
@@ -7729,19 +7720,19 @@
         <v>673</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>359</v>
+        <v>674</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G160" s="1" t="s">
         <v>15</v>
@@ -7755,22 +7746,22 @@
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>677</v>
+        <v>104</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="G161" s="1" t="s">
         <v>15</v>
@@ -7784,22 +7775,22 @@
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>104</v>
+        <v>682</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="F162" s="1" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="G162" s="1" t="s">
         <v>15</v>
@@ -7813,28 +7804,28 @@
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>685</v>
+        <v>359</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="G163" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H163" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I163" s="6">
         <v>46118.568367997686</v>
@@ -7842,28 +7833,28 @@
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>359</v>
+        <v>691</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="G164" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I164" s="6">
         <v>46118.568367997686</v>
@@ -7871,22 +7862,22 @@
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="G165" s="1" t="s">
         <v>15</v>
@@ -7900,22 +7891,22 @@
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G166" s="1" t="s">
         <v>15</v>
@@ -7929,22 +7920,22 @@
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D167" s="1" t="s">
-        <v>690</v>
+        <v>704</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="G167" s="1" t="s">
         <v>15</v>
@@ -7958,25 +7949,25 @@
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G168" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H168" s="1" t="s">
         <v>15</v>
@@ -7987,25 +7978,25 @@
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>711</v>
+        <v>262</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D169" s="1" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="F169" s="1" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="G169" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H169" s="1" t="s">
         <v>15</v>
@@ -8016,19 +8007,19 @@
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>262</v>
+        <v>716</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>717</v>
@@ -8054,16 +8045,16 @@
         <v>11</v>
       </c>
       <c r="D171" s="1" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="F171" s="1" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="G171" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H171" s="1" t="s">
         <v>15</v>
@@ -8074,25 +8065,25 @@
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D172" s="1" t="s">
-        <v>715</v>
+        <v>724</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="G172" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H172" s="1" t="s">
         <v>15</v>
@@ -8103,22 +8094,22 @@
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D173" s="1" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="F173" s="1" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="G173" s="1" t="s">
         <v>15</v>
@@ -8132,16 +8123,16 @@
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>731</v>
+        <v>180</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="E174" s="1" t="s">
         <v>732</v>
@@ -8164,13 +8155,13 @@
         <v>734</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="E175" s="1" t="s">
         <v>735</v>
@@ -8193,19 +8184,19 @@
         <v>737</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>167</v>
+        <v>738</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D176" s="1" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="E176" s="1" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F176" s="1" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G176" s="1" t="s">
         <v>15</v>
@@ -8219,22 +8210,22 @@
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D177" s="1" t="s">
-        <v>727</v>
+        <v>743</v>
       </c>
       <c r="E177" s="1" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="G177" s="1" t="s">
         <v>15</v>
@@ -8248,22 +8239,22 @@
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="E178" s="1" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="G178" s="1" t="s">
         <v>15</v>
@@ -8277,25 +8268,25 @@
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="E179" s="1" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="F179" s="1" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="G179" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H179" s="1" t="s">
         <v>15</v>
@@ -8306,25 +8297,25 @@
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D180" s="1" t="s">
-        <v>746</v>
+        <v>756</v>
       </c>
       <c r="E180" s="1" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="G180" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H180" s="1" t="s">
         <v>15</v>
@@ -8335,25 +8326,25 @@
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="E181" s="1" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="G181" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H181" s="1" t="s">
         <v>15</v>
@@ -8364,25 +8355,25 @@
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>763</v>
+        <v>171</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D182" s="1" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="E182" s="1" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="F182" s="1" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="G182" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H182" s="1" t="s">
         <v>15</v>
@@ -8393,25 +8384,25 @@
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>171</v>
+        <v>768</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D183" s="1" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="E183" s="1" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="F183" s="1" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="G183" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H183" s="1" t="s">
         <v>15</v>
@@ -8422,25 +8413,25 @@
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>771</v>
+        <v>359</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="D184" s="1" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="E184" s="1" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="F184" s="1" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="G184" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H184" s="1" t="s">
         <v>15</v>
@@ -8449,38 +8440,9 @@
         <v>46118.568367997686</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A185" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="B185" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="C185" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D185" s="1" t="s">
-        <v>775</v>
-      </c>
-      <c r="E185" s="1" t="s">
-        <v>776</v>
-      </c>
-      <c r="F185" s="1" t="s">
-        <v>777</v>
-      </c>
-      <c r="G185" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H185" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I185" s="6">
-        <v>46118.568367997686</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H185">
-    <sortCondition ref="D2:D185"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H184">
+    <sortCondition ref="D2:D184"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -8491,18 +8453,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21065E3C-A718-4C68-867F-24F90DCB0AB2}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8511,7 +8473,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -8546,7 +8508,7 @@
         <v>383</v>
       </c>
       <c r="C2" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="D2" t="s">
         <v>23</v>
@@ -8567,6 +8529,38 @@
         <v>20</v>
       </c>
       <c r="J2" s="6">
+        <v>46119.568368055552</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C3" t="s">
+        <v>531</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="6">
         <v>46119.568368055552</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish for updated membership directory 	modified:   .quarto/idx/index.qmd.json 	modified:   .quarto/preview/lock 	modified:   README.md 	modified:   _site/site_libs/quarto-html/quarto.js 	modified:   _site/site_libs/quarto-search/quarto-search.js 	modified:   documents/CCPRO_Membership_Database.xlsx
</commit_message>
<xml_diff>
--- a/documents/CCPRO_Membership_Database.xlsx
+++ b/documents/CCPRO_Membership_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hcc365-my.sharepoint.com/personal/rking3387_haywood_edu/Documents/LK-Obsidian/1_Projects/3_Non-Data Projects/CCPRO-Website/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{2365E0E2-A4E4-410D-B773-CA0E0058FBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CEBE380-80EE-4B1C-9794-EE64B8530724}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{B2A14708-9D94-45B4-90C6-CB38EABA9F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6D25EAA-1C01-493F-B369-8C97ECA1D681}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{AB234C9B-704F-466F-A7C7-F848F51275B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{AB234C9B-704F-466F-A7C7-F848F51275B9}"/>
   </bookViews>
   <sheets>
     <sheet name="New Membership" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1500" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="795">
   <si>
     <t>current_member_name</t>
   </si>
@@ -1632,9 +1632,18 @@
     <t>hunter.ashworth@piedmontcc.edu</t>
   </si>
   <si>
+    <t>Michele Mathis</t>
+  </si>
+  <si>
     <t>Director, Research and Institutional Effectiveness</t>
   </si>
   <si>
+    <t>336-322-2237</t>
+  </si>
+  <si>
+    <t>Michele.Mathis@piedmontcc.edu</t>
+  </si>
+  <si>
     <t>Dr. Brandy Leder</t>
   </si>
   <si>
@@ -2364,17 +2373,62 @@
     <t>bwallace@wilsoncc.edu</t>
   </si>
   <si>
+    <t>Angela Gates Daquila</t>
+  </si>
+  <si>
+    <t>Nursing Instructor</t>
+  </si>
+  <si>
+    <t> 407-462-1234</t>
+  </si>
+  <si>
+    <t>agatesdaquila130@nashcc.edu</t>
+  </si>
+  <si>
+    <t>Emily Smail</t>
+  </si>
+  <si>
+    <t>Director of Research and Evaluation</t>
+  </si>
+  <si>
+    <t>919-807-7024</t>
+  </si>
+  <si>
+    <t>smaile@nccommunitycolleges.edu</t>
+  </si>
+  <si>
+    <t>Amanda Spangle</t>
+  </si>
+  <si>
+    <t>Data &amp; Reporting Specialist</t>
+  </si>
+  <si>
+    <t>704-216-3692</t>
+  </si>
+  <si>
+    <t>amanda.spangle@rccc.edu</t>
+  </si>
+  <si>
+    <t>Logan Okun</t>
+  </si>
+  <si>
+    <t>Senior Director of Marketing &amp; Communications</t>
+  </si>
+  <si>
+    <t>252-515-6934</t>
+  </si>
+  <si>
+    <t>loganl4449@carteret.edu</t>
+  </si>
+  <si>
     <t>updated_name</t>
-  </si>
-  <si>
-    <t>Assessment &amp; Research Analyst</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2399,14 +2453,6 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2466,9 +2512,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2477,14 +2522,51 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="13">
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2666,63 +2748,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="27" formatCode="m/d/yyyy\ h:mm"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2737,26 +2762,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}" name="Table1" displayName="Table1" ref="A1:I184" totalsRowShown="0" dataDxfId="9">
-  <autoFilter ref="A1:I184" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}" name="Table1" displayName="Table1" ref="A1:I189" totalsRowShown="0" dataDxfId="12">
+  <autoFilter ref="A1:I189" xr:uid="{54B221D3-A8CB-48C6-9327-2D1014AF80DE}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{3F4788B0-7800-4F61-A6A0-0A5282B58274}" name="current_member_name" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{7F07D569-61A9-4190-B534-F0A0ED69069B}" name="title" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{9886F57E-D00C-4B9F-A0C2-68AE44FFB1C1}" name="region" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{43D32C3F-222C-4E2F-80E3-A64452A9954E}" name="college" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{322F794B-2038-47B1-9E2D-C1547157662B}" name="college_phone" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{C85BF0CF-7B73-4382-B1BD-709C682A5F5E}" name="email" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{AD8863AA-BC53-493D-8F4B-50F6297D8363}" name="sacscoc_liaison" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{9D36408C-FDDB-47CD-ADF3-3D3423E576E5}" name="executive_committee_member" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{0F49363C-D270-48A5-9781-7164FAE388B6}" name="date_submitted" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{3F4788B0-7800-4F61-A6A0-0A5282B58274}" name="current_member_name" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{7F07D569-61A9-4190-B534-F0A0ED69069B}" name="title" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9886F57E-D00C-4B9F-A0C2-68AE44FFB1C1}" name="region" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{43D32C3F-222C-4E2F-80E3-A64452A9954E}" name="college" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{322F794B-2038-47B1-9E2D-C1547157662B}" name="college_phone" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{C85BF0CF-7B73-4382-B1BD-709C682A5F5E}" name="email" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{AD8863AA-BC53-493D-8F4B-50F6297D8363}" name="sacscoc_liaison" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{9D36408C-FDDB-47CD-ADF3-3D3423E576E5}" name="executive_committee_member" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{0F49363C-D270-48A5-9781-7164FAE388B6}" name="date_submitted" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}" name="Table2" displayName="Table2" ref="A1:J3" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
-  <autoFilter ref="A1:J3" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}" name="Table2" displayName="Table2" ref="A1:J2" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:J2" xr:uid="{61B4CCE7-16F1-4E8B-8802-7FC1F5B29E29}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1958840C-24FF-4B93-989A-E3D4C45B1A63}" name="current_member_name"/>
     <tableColumn id="2" xr3:uid="{901C16ED-C9F3-4383-BD31-77D387CB8D82}" name="updated_name"/>
@@ -2764,10 +2789,10 @@
     <tableColumn id="4" xr3:uid="{D537AEE6-D7E8-42C2-A888-27F2620BC4AD}" name="region"/>
     <tableColumn id="5" xr3:uid="{0BE7D98F-B4E1-4E8D-9DF5-E6F4A6853C3E}" name="college"/>
     <tableColumn id="6" xr3:uid="{1D6C305C-76DF-4821-81ED-060BAA652553}" name="college_phone"/>
-    <tableColumn id="7" xr3:uid="{385958E6-6FB8-4783-8FE2-082ADA0EB4BA}" name="email" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{385958E6-6FB8-4783-8FE2-082ADA0EB4BA}" name="email"/>
     <tableColumn id="8" xr3:uid="{00D30660-3FCE-44C9-AB93-4E03423B4D57}" name="sacscoc_liaison"/>
     <tableColumn id="9" xr3:uid="{01985461-802C-412E-B311-CF5D8C545457}" name="executive_committee_member"/>
-    <tableColumn id="10" xr3:uid="{57C737E1-2C3F-49A2-82FB-808C0E64D264}" name="date_submitted" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{57C737E1-2C3F-49A2-82FB-808C0E64D264}" name="date_submitted"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3090,7 +3115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4617D616-0D58-46B6-AC53-2FFE73FE93B0}">
-  <dimension ref="A1:I184"/>
+  <dimension ref="A1:I189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -3158,7 +3183,7 @@
       <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="7">
         <v>46118.568368055552</v>
       </c>
     </row>
@@ -3187,7 +3212,7 @@
       <c r="H3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="7">
         <v>46118.568368055552</v>
       </c>
     </row>
@@ -3216,7 +3241,7 @@
       <c r="H4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3245,7 +3270,7 @@
       <c r="H5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3274,7 +3299,7 @@
       <c r="H6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3303,7 +3328,7 @@
       <c r="H7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3332,7 +3357,7 @@
       <c r="H8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3361,7 +3386,7 @@
       <c r="H9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3390,7 +3415,7 @@
       <c r="H10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3419,7 +3444,7 @@
       <c r="H11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3448,7 +3473,7 @@
       <c r="H12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3477,7 +3502,7 @@
       <c r="H13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3506,7 +3531,7 @@
       <c r="H14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3535,7 +3560,7 @@
       <c r="H15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3564,7 +3589,7 @@
       <c r="H16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3593,7 +3618,7 @@
       <c r="H17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3622,7 +3647,7 @@
       <c r="H18" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3651,7 +3676,7 @@
       <c r="H19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3680,7 +3705,7 @@
       <c r="H20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3709,7 +3734,7 @@
       <c r="H21" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3738,7 +3763,7 @@
       <c r="H22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3767,7 +3792,7 @@
       <c r="H23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3796,7 +3821,7 @@
       <c r="H24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3825,7 +3850,7 @@
       <c r="H25" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3854,7 +3879,7 @@
       <c r="H26" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3883,7 +3908,7 @@
       <c r="H27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3912,7 +3937,7 @@
       <c r="H28" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3941,7 +3966,7 @@
       <c r="H29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3970,7 +3995,7 @@
       <c r="H30" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -3999,7 +4024,7 @@
       <c r="H31" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4028,7 +4053,7 @@
       <c r="H32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4057,7 +4082,7 @@
       <c r="H33" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4086,7 +4111,7 @@
       <c r="H34" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I34" s="6">
+      <c r="I34" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4115,7 +4140,7 @@
       <c r="H35" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I35" s="6">
+      <c r="I35" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4144,7 +4169,7 @@
       <c r="H36" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4173,7 +4198,7 @@
       <c r="H37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I37" s="6">
+      <c r="I37" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4202,7 +4227,7 @@
       <c r="H38" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4231,7 +4256,7 @@
       <c r="H39" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I39" s="6">
+      <c r="I39" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4260,7 +4285,7 @@
       <c r="H40" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="6">
+      <c r="I40" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4289,7 +4314,7 @@
       <c r="H41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I41" s="6">
+      <c r="I41" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4318,7 +4343,7 @@
       <c r="H42" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I42" s="6">
+      <c r="I42" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4347,7 +4372,7 @@
       <c r="H43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I43" s="6">
+      <c r="I43" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4376,7 +4401,7 @@
       <c r="H44" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I44" s="6">
+      <c r="I44" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4405,7 +4430,7 @@
       <c r="H45" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I45" s="6">
+      <c r="I45" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4434,7 +4459,7 @@
       <c r="H46" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I46" s="6">
+      <c r="I46" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4463,7 +4488,7 @@
       <c r="H47" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I47" s="6">
+      <c r="I47" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4492,7 +4517,7 @@
       <c r="H48" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I48" s="6">
+      <c r="I48" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4521,7 +4546,7 @@
       <c r="H49" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I49" s="6">
+      <c r="I49" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4550,7 +4575,7 @@
       <c r="H50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I50" s="6">
+      <c r="I50" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4579,7 +4604,7 @@
       <c r="H51" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I51" s="6">
+      <c r="I51" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4608,7 +4633,7 @@
       <c r="H52" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I52" s="6">
+      <c r="I52" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4637,7 +4662,7 @@
       <c r="H53" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I53" s="6">
+      <c r="I53" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4666,7 +4691,7 @@
       <c r="H54" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I54" s="6">
+      <c r="I54" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4695,7 +4720,7 @@
       <c r="H55" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I55" s="6">
+      <c r="I55" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4724,7 +4749,7 @@
       <c r="H56" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I56" s="6">
+      <c r="I56" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4753,7 +4778,7 @@
       <c r="H57" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I57" s="6">
+      <c r="I57" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4782,7 +4807,7 @@
       <c r="H58" t="s">
         <v>15</v>
       </c>
-      <c r="I58" s="6">
+      <c r="I58" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4811,7 +4836,7 @@
       <c r="H59" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I59" s="6">
+      <c r="I59" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4840,7 +4865,7 @@
       <c r="H60" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I60" s="6">
+      <c r="I60" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4869,7 +4894,7 @@
       <c r="H61" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I61" s="6">
+      <c r="I61" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4898,7 +4923,7 @@
       <c r="H62" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I62" s="6">
+      <c r="I62" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4927,7 +4952,7 @@
       <c r="H63" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I63" s="6">
+      <c r="I63" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4956,7 +4981,7 @@
       <c r="H64" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I64" s="6">
+      <c r="I64" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -4985,7 +5010,7 @@
       <c r="H65" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I65" s="6">
+      <c r="I65" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5014,7 +5039,7 @@
       <c r="H66" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I66" s="6">
+      <c r="I66" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5043,7 +5068,7 @@
       <c r="H67" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I67" s="6">
+      <c r="I67" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5072,7 +5097,7 @@
       <c r="H68" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I68" s="6">
+      <c r="I68" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5101,7 +5126,7 @@
       <c r="H69" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I69" s="6">
+      <c r="I69" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5130,7 +5155,7 @@
       <c r="H70" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I70" s="6">
+      <c r="I70" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5159,7 +5184,7 @@
       <c r="H71" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I71" s="6">
+      <c r="I71" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5188,7 +5213,7 @@
       <c r="H72" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I72" s="6">
+      <c r="I72" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5217,7 +5242,7 @@
       <c r="H73" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I73" s="6">
+      <c r="I73" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5246,7 +5271,7 @@
       <c r="H74" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I74" s="6">
+      <c r="I74" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5275,7 +5300,7 @@
       <c r="H75" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I75" s="6">
+      <c r="I75" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5304,7 +5329,7 @@
       <c r="H76" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I76" s="6">
+      <c r="I76" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5333,7 +5358,7 @@
       <c r="H77" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I77" s="6">
+      <c r="I77" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5362,7 +5387,7 @@
       <c r="H78" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I78" s="6">
+      <c r="I78" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5391,7 +5416,7 @@
       <c r="H79" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I79" s="6">
+      <c r="I79" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5420,7 +5445,7 @@
       <c r="H80" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I80" s="6">
+      <c r="I80" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5449,7 +5474,7 @@
       <c r="H81" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I81" s="6">
+      <c r="I81" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5478,7 +5503,7 @@
       <c r="H82" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I82" s="6">
+      <c r="I82" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5507,7 +5532,7 @@
       <c r="H83" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I83" s="6">
+      <c r="I83" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5536,7 +5561,7 @@
       <c r="H84" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I84" s="6">
+      <c r="I84" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5565,7 +5590,7 @@
       <c r="H85" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I85" s="6">
+      <c r="I85" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5594,7 +5619,7 @@
       <c r="H86" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I86" s="6">
+      <c r="I86" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5623,7 +5648,7 @@
       <c r="H87" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I87" s="6">
+      <c r="I87" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5652,7 +5677,7 @@
       <c r="H88" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I88" s="6">
+      <c r="I88" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5681,7 +5706,7 @@
       <c r="H89" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I89" s="6">
+      <c r="I89" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5710,7 +5735,7 @@
       <c r="H90" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I90" s="6">
+      <c r="I90" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5739,7 +5764,7 @@
       <c r="H91" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I91" s="6">
+      <c r="I91" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5768,7 +5793,7 @@
       <c r="H92" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I92" s="6">
+      <c r="I92" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5797,7 +5822,7 @@
       <c r="H93" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I93" s="6">
+      <c r="I93" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5826,7 +5851,7 @@
       <c r="H94" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I94" s="6">
+      <c r="I94" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5855,7 +5880,7 @@
       <c r="H95" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I95" s="6">
+      <c r="I95" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5884,7 +5909,7 @@
       <c r="H96" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I96" s="6">
+      <c r="I96" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5913,7 +5938,7 @@
       <c r="H97" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I97" s="6">
+      <c r="I97" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5942,7 +5967,7 @@
       <c r="H98" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I98" s="6">
+      <c r="I98" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -5971,7 +5996,7 @@
       <c r="H99" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I99" s="6">
+      <c r="I99" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6000,7 +6025,7 @@
       <c r="H100" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I100" s="6">
+      <c r="I100" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6029,7 +6054,7 @@
       <c r="H101" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I101" s="6">
+      <c r="I101" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6058,7 +6083,7 @@
       <c r="H102" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I102" s="6">
+      <c r="I102" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6087,7 +6112,7 @@
       <c r="H103" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I103" s="6">
+      <c r="I103" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6116,7 +6141,7 @@
       <c r="H104" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I104" s="6">
+      <c r="I104" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6145,7 +6170,7 @@
       <c r="H105" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I105" s="6">
+      <c r="I105" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6174,7 +6199,7 @@
       <c r="H106" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I106" s="6">
+      <c r="I106" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6203,7 +6228,7 @@
       <c r="H107" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I107" s="6">
+      <c r="I107" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6232,7 +6257,7 @@
       <c r="H108" t="s">
         <v>15</v>
       </c>
-      <c r="I108" s="6">
+      <c r="I108" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6261,7 +6286,7 @@
       <c r="H109" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I109" s="6">
+      <c r="I109" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6290,7 +6315,7 @@
       <c r="H110" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I110" s="6">
+      <c r="I110" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6319,7 +6344,7 @@
       <c r="H111" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I111" s="6">
+      <c r="I111" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6348,7 +6373,7 @@
       <c r="H112" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I112" s="6">
+      <c r="I112" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6377,7 +6402,7 @@
       <c r="H113" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I113" s="6">
+      <c r="I113" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6406,7 +6431,7 @@
       <c r="H114" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I114" s="6">
+      <c r="I114" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6435,7 +6460,7 @@
       <c r="H115" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I115" s="6">
+      <c r="I115" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6464,7 +6489,7 @@
       <c r="H116" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I116" s="6">
+      <c r="I116" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6493,7 +6518,7 @@
       <c r="H117" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I117" s="6">
+      <c r="I117" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6522,7 +6547,7 @@
       <c r="H118" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I118" s="6">
+      <c r="I118" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6551,7 +6576,7 @@
       <c r="H119" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I119" s="6">
+      <c r="I119" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6580,7 +6605,7 @@
       <c r="H120" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I120" s="6">
+      <c r="I120" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6609,7 +6634,7 @@
       <c r="H121" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I121" s="6">
+      <c r="I121" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6638,7 +6663,7 @@
       <c r="H122" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I122" s="6">
+      <c r="I122" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6667,7 +6692,7 @@
       <c r="H123" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I123" s="6">
+      <c r="I123" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6696,7 +6721,7 @@
       <c r="H124" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I124" s="6">
+      <c r="I124" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6725,173 +6750,173 @@
       <c r="H125" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I125" s="6">
+      <c r="I125" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B126" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="C126" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="E126" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="C126" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D126" s="1" t="s">
+      <c r="F126" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="E126" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="F126" s="1" t="s">
-        <v>536</v>
-      </c>
       <c r="G126" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H126" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I126" s="6">
+      <c r="I126" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="E127" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="F127" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="F127" s="1" t="s">
-        <v>540</v>
-      </c>
       <c r="G127" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I127" s="6">
+        <v>15</v>
+      </c>
+      <c r="I127" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="B128" s="1" t="s">
         <v>541</v>
-      </c>
-      <c r="B128" s="1" t="s">
-        <v>542</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E128" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="F128" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="F128" s="1" t="s">
-        <v>544</v>
-      </c>
       <c r="G128" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I128" s="6">
+        <v>20</v>
+      </c>
+      <c r="I128" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="B129" s="1" t="s">
         <v>545</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>546</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E129" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="F129" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="F129" s="1" t="s">
-        <v>548</v>
-      </c>
       <c r="G129" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H129" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I129" s="6">
+      <c r="I129" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B130" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="B130" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="C130" s="1" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D130" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="E130" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="E130" s="1" t="s">
+      <c r="F130" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="F130" s="1" t="s">
-        <v>552</v>
-      </c>
       <c r="G130" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H130" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I130" s="6">
+      <c r="I130" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>554</v>
+        <v>104</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="E131" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="F131" s="1" t="s">
         <v>555</v>
-      </c>
-      <c r="F131" s="1" t="s">
-        <v>556</v>
       </c>
       <c r="G131" s="1" t="s">
         <v>20</v>
@@ -6899,36 +6924,36 @@
       <c r="H131" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I131" s="6">
+      <c r="I131" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="B132" s="1" t="s">
         <v>557</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>558</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>559</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H132" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I132" s="6">
+      <c r="I132" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -6937,172 +6962,172 @@
         <v>560</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>359</v>
+        <v>561</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="E133" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="F133" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="F133" s="1" t="s">
-        <v>563</v>
-      </c>
       <c r="G133" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H133" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I133" s="6">
+      <c r="I133" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>565</v>
+        <v>359</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="E134" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="F134" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="F134" s="1" t="s">
-        <v>567</v>
-      </c>
       <c r="G134" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H134" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I134" s="6">
+      <c r="I134" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B135" s="1" t="s">
         <v>568</v>
-      </c>
-      <c r="B135" s="1" t="s">
-        <v>569</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="E135" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="F135" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="F135" s="1" t="s">
-        <v>571</v>
-      </c>
       <c r="G135" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H135" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I135" s="6">
+      <c r="I135" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B136" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="C136" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="E136" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="C136" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D136" s="1" t="s">
+      <c r="F136" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="E136" s="1" t="s">
-        <v>575</v>
-      </c>
-      <c r="F136" s="1" t="s">
-        <v>576</v>
-      </c>
       <c r="G136" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H136" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I136" s="6">
+      <c r="I136" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D137" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="E137" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="C137" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D137" s="1" t="s">
+      <c r="F137" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="E137" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="F137" s="1" t="s">
-        <v>581</v>
-      </c>
       <c r="G137" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H137" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I137" s="6">
+      <c r="I137" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>584</v>
       </c>
       <c r="G138" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H138" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I138" s="6">
+      <c r="I138" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -7117,384 +7142,384 @@
         <v>11</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E139" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="F139" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="F139" s="1" t="s">
-        <v>588</v>
-      </c>
       <c r="G139" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H139" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I139" s="6">
+      <c r="I139" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="B140" s="1" t="s">
         <v>589</v>
-      </c>
-      <c r="B140" s="1" t="s">
-        <v>590</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D140" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="F140" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="E140" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="F140" s="1" t="s">
-        <v>593</v>
-      </c>
       <c r="G140" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H140" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I140" s="6">
+      <c r="I140" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E141" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="F141" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="F141" s="1" t="s">
-        <v>597</v>
-      </c>
       <c r="G141" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H141" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I141" s="6">
+        <v>15</v>
+      </c>
+      <c r="I141" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B142" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="C142" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="E142" s="1" t="s">
         <v>599</v>
       </c>
-      <c r="C142" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D142" s="1" t="s">
+      <c r="F142" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="E142" s="1" t="s">
-        <v>601</v>
-      </c>
-      <c r="F142" s="1" t="s">
-        <v>602</v>
-      </c>
       <c r="G142" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H142" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I142" s="6">
+        <v>20</v>
+      </c>
+      <c r="I142" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E143" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="F143" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="F143" s="1" t="s">
-        <v>606</v>
-      </c>
       <c r="G143" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H143" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I143" s="6">
+      <c r="I143" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="B144" s="1" t="s">
         <v>607</v>
-      </c>
-      <c r="B144" s="1" t="s">
-        <v>608</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E144" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="F144" s="1" t="s">
         <v>609</v>
       </c>
-      <c r="F144" s="1" t="s">
-        <v>610</v>
-      </c>
       <c r="G144" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H144" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I144" s="6">
+      <c r="I144" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="B145" s="1" t="s">
         <v>611</v>
-      </c>
-      <c r="B145" s="1" t="s">
-        <v>612</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E145" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="F145" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="F145" s="1" t="s">
-        <v>614</v>
-      </c>
       <c r="G145" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H145" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I145" s="6">
+      <c r="I145" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="B146" s="1" t="s">
         <v>615</v>
-      </c>
-      <c r="B146" s="1" t="s">
-        <v>616</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E146" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="F146" s="1" t="s">
         <v>617</v>
       </c>
-      <c r="F146" s="1" t="s">
-        <v>618</v>
-      </c>
       <c r="G146" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H146" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I146" s="6">
+      <c r="I146" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="B147" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="C147" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="E147" s="1" t="s">
         <v>620</v>
       </c>
-      <c r="C147" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D147" s="1" t="s">
+      <c r="F147" s="1" t="s">
         <v>621</v>
       </c>
-      <c r="E147" s="1" t="s">
-        <v>622</v>
-      </c>
-      <c r="F147" s="1" t="s">
-        <v>623</v>
-      </c>
       <c r="G147" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H147" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I147" s="6">
+      <c r="I147" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E148" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="F148" s="1" t="s">
         <v>626</v>
       </c>
-      <c r="F148" s="1" t="s">
-        <v>627</v>
-      </c>
       <c r="G148" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H148" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I148" s="6">
+      <c r="I148" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="B149" s="1" t="s">
         <v>628</v>
-      </c>
-      <c r="B149" s="1" t="s">
-        <v>629</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E149" s="1" t="s">
+        <v>629</v>
+      </c>
+      <c r="F149" s="1" t="s">
         <v>630</v>
       </c>
-      <c r="F149" s="1" t="s">
-        <v>631</v>
-      </c>
       <c r="G149" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H149" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I149" s="6">
+      <c r="I149" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="B150" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="C150" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="E150" s="1" t="s">
         <v>633</v>
       </c>
-      <c r="C150" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D150" s="1" t="s">
+      <c r="F150" s="1" t="s">
         <v>634</v>
       </c>
-      <c r="E150" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="F150" s="1" t="s">
-        <v>636</v>
-      </c>
       <c r="G150" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H150" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I150" s="6">
+      <c r="I150" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E151" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="F151" s="1" t="s">
         <v>639</v>
       </c>
-      <c r="F151" s="1" t="s">
-        <v>640</v>
-      </c>
       <c r="G151" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H151" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I151" s="6">
+      <c r="I151" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="B152" s="1" t="s">
         <v>641</v>
-      </c>
-      <c r="B152" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E152" s="1" t="s">
         <v>642</v>
@@ -7508,7 +7533,7 @@
       <c r="H152" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I152" s="6">
+      <c r="I152" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -7517,129 +7542,129 @@
         <v>644</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>645</v>
+        <v>171</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D153" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="F153" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="E153" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="F153" s="1" t="s">
-        <v>648</v>
-      </c>
       <c r="G153" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H153" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I153" s="6">
+      <c r="I153" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E154" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="F154" s="1" t="s">
         <v>651</v>
       </c>
-      <c r="F154" s="1" t="s">
-        <v>652</v>
-      </c>
       <c r="G154" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H154" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I154" s="6">
+      <c r="I154" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
+        <v>652</v>
+      </c>
+      <c r="B155" s="1" t="s">
         <v>653</v>
-      </c>
-      <c r="B155" s="1" t="s">
-        <v>654</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E155" s="1" t="s">
+        <v>654</v>
+      </c>
+      <c r="F155" s="1" t="s">
         <v>655</v>
       </c>
-      <c r="F155" s="1" t="s">
-        <v>656</v>
-      </c>
       <c r="G155" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H155" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I155" s="6">
+      <c r="I155" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B156" s="1" t="s">
         <v>657</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="C156" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D156" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="E156" s="1" t="s">
         <v>658</v>
       </c>
-      <c r="C156" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D156" s="1" t="s">
+      <c r="F156" s="1" t="s">
         <v>659</v>
       </c>
-      <c r="E156" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="F156" s="1" t="s">
-        <v>661</v>
-      </c>
       <c r="G156" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H156" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I156" s="6">
+      <c r="I156" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>36</v>
+        <v>661</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="E157" s="1" t="s">
         <v>663</v>
@@ -7648,12 +7673,12 @@
         <v>664</v>
       </c>
       <c r="G157" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H157" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I157" s="6">
+      <c r="I157" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -7662,42 +7687,42 @@
         <v>665</v>
       </c>
       <c r="B158" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="E158" s="1" t="s">
         <v>666</v>
       </c>
-      <c r="C158" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D158" s="1" t="s">
+      <c r="F158" s="1" t="s">
         <v>667</v>
       </c>
-      <c r="E158" s="1" t="s">
-        <v>668</v>
-      </c>
-      <c r="F158" s="1" t="s">
-        <v>669</v>
-      </c>
       <c r="G158" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H158" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I158" s="6">
+      <c r="I158" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>359</v>
+        <v>669</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="E159" s="1" t="s">
         <v>671</v>
@@ -7711,7 +7736,7 @@
       <c r="H159" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I159" s="6">
+      <c r="I159" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -7720,306 +7745,306 @@
         <v>673</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>674</v>
+        <v>359</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="E160" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="F160" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="F160" s="1" t="s">
-        <v>676</v>
-      </c>
       <c r="G160" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H160" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I160" s="6">
+      <c r="I160" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="B161" s="1" t="s">
         <v>677</v>
       </c>
-      <c r="B161" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="C161" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D161" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="E161" s="1" t="s">
         <v>678</v>
       </c>
-      <c r="E161" s="1" t="s">
+      <c r="F161" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="F161" s="1" t="s">
-        <v>680</v>
-      </c>
       <c r="G161" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H161" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I161" s="6">
+      <c r="I161" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>682</v>
+        <v>104</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D162" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="E162" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="F162" s="1" t="s">
         <v>683</v>
       </c>
-      <c r="E162" s="1" t="s">
-        <v>684</v>
-      </c>
-      <c r="F162" s="1" t="s">
-        <v>685</v>
-      </c>
       <c r="G162" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H162" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I162" s="6">
+      <c r="I162" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D163" s="1" t="s">
         <v>686</v>
       </c>
-      <c r="B163" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="C163" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D163" s="1" t="s">
+      <c r="E163" s="1" t="s">
         <v>687</v>
       </c>
-      <c r="E163" s="1" t="s">
+      <c r="F163" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="F163" s="1" t="s">
-        <v>689</v>
-      </c>
       <c r="G163" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H163" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I163" s="6">
+        <v>15</v>
+      </c>
+      <c r="I163" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>691</v>
+        <v>359</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="E164" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="F164" s="1" t="s">
         <v>692</v>
       </c>
-      <c r="F164" s="1" t="s">
-        <v>693</v>
-      </c>
       <c r="G164" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I164" s="6">
+        <v>20</v>
+      </c>
+      <c r="I164" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="B165" s="1" t="s">
         <v>694</v>
-      </c>
-      <c r="B165" s="1" t="s">
-        <v>695</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="E165" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="F165" s="1" t="s">
         <v>696</v>
       </c>
-      <c r="F165" s="1" t="s">
-        <v>697</v>
-      </c>
       <c r="G165" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H165" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I165" s="6">
+      <c r="I165" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="B166" s="1" t="s">
         <v>698</v>
-      </c>
-      <c r="B166" s="1" t="s">
-        <v>699</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="E166" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="F166" s="1" t="s">
         <v>700</v>
       </c>
-      <c r="F166" s="1" t="s">
-        <v>701</v>
-      </c>
       <c r="G166" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H166" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I166" s="6">
+      <c r="I166" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B167" s="1" t="s">
         <v>702</v>
-      </c>
-      <c r="B167" s="1" t="s">
-        <v>703</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D167" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="F167" s="1" t="s">
         <v>704</v>
       </c>
-      <c r="E167" s="1" t="s">
-        <v>705</v>
-      </c>
-      <c r="F167" s="1" t="s">
-        <v>706</v>
-      </c>
       <c r="G167" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H167" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I167" s="6">
+      <c r="I167" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E168" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="F168" s="1" t="s">
         <v>709</v>
       </c>
-      <c r="F168" s="1" t="s">
-        <v>710</v>
-      </c>
       <c r="G168" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H168" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I168" s="6">
+      <c r="I168" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="B169" s="1" t="s">
         <v>711</v>
       </c>
-      <c r="B169" s="1" t="s">
-        <v>262</v>
-      </c>
       <c r="C169" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D169" s="1" t="s">
+        <v>707</v>
+      </c>
+      <c r="E169" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="E169" s="1" t="s">
+      <c r="F169" s="1" t="s">
         <v>713</v>
       </c>
-      <c r="F169" s="1" t="s">
-        <v>714</v>
-      </c>
       <c r="G169" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H169" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I169" s="6">
+      <c r="I169" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>716</v>
+        <v>262</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>717</v>
@@ -8030,7 +8055,7 @@
       <c r="H170" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I170" s="6">
+      <c r="I170" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -8045,94 +8070,94 @@
         <v>11</v>
       </c>
       <c r="D171" s="1" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="E171" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="F171" s="1" t="s">
         <v>720</v>
       </c>
-      <c r="F171" s="1" t="s">
-        <v>721</v>
-      </c>
       <c r="G171" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H171" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I171" s="6">
+      <c r="I171" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="B172" s="1" t="s">
         <v>722</v>
-      </c>
-      <c r="B172" s="1" t="s">
-        <v>723</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D172" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="E172" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="F172" s="1" t="s">
         <v>724</v>
       </c>
-      <c r="E172" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="F172" s="1" t="s">
-        <v>726</v>
-      </c>
       <c r="G172" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H172" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I172" s="6">
+      <c r="I172" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D173" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="E173" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="F173" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="F173" s="1" t="s">
-        <v>730</v>
-      </c>
       <c r="G173" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H173" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I173" s="6">
+      <c r="I173" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="B174" s="1" t="s">
         <v>731</v>
-      </c>
-      <c r="B174" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="E174" s="1" t="s">
         <v>732</v>
@@ -8146,7 +8171,7 @@
       <c r="H174" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I174" s="6">
+      <c r="I174" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -8155,13 +8180,13 @@
         <v>734</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="E175" s="1" t="s">
         <v>735</v>
@@ -8175,7 +8200,7 @@
       <c r="H175" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I175" s="6">
+      <c r="I175" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
@@ -8184,265 +8209,408 @@
         <v>737</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>738</v>
+        <v>167</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D176" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="E176" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="F176" s="1" t="s">
         <v>739</v>
       </c>
-      <c r="F176" s="1" t="s">
-        <v>740</v>
-      </c>
       <c r="G176" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H176" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I176" s="6">
+      <c r="I176" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="B177" s="1" t="s">
         <v>741</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="C177" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D177" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="E177" s="1" t="s">
         <v>742</v>
       </c>
-      <c r="C177" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D177" s="1" t="s">
+      <c r="F177" s="1" t="s">
         <v>743</v>
       </c>
-      <c r="E177" s="1" t="s">
-        <v>744</v>
-      </c>
-      <c r="F177" s="1" t="s">
-        <v>745</v>
-      </c>
       <c r="G177" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H177" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I177" s="6">
+      <c r="I177" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="E178" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="F178" s="1" t="s">
         <v>748</v>
       </c>
-      <c r="F178" s="1" t="s">
-        <v>749</v>
-      </c>
       <c r="G178" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H178" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I178" s="6">
+      <c r="I178" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="B179" s="1" t="s">
         <v>750</v>
-      </c>
-      <c r="B179" s="1" t="s">
-        <v>751</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="E179" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="F179" s="1" t="s">
         <v>752</v>
       </c>
-      <c r="F179" s="1" t="s">
-        <v>753</v>
-      </c>
       <c r="G179" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H179" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I179" s="6">
+      <c r="I179" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="B180" s="1" t="s">
         <v>754</v>
       </c>
-      <c r="B180" s="1" t="s">
+      <c r="C180" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D180" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="E180" s="1" t="s">
         <v>755</v>
       </c>
-      <c r="C180" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D180" s="1" t="s">
+      <c r="F180" s="1" t="s">
         <v>756</v>
       </c>
-      <c r="E180" s="1" t="s">
-        <v>757</v>
-      </c>
-      <c r="F180" s="1" t="s">
-        <v>758</v>
-      </c>
       <c r="G180" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H180" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I180" s="6">
+      <c r="I180" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="E181" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="F181" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="F181" s="1" t="s">
-        <v>762</v>
-      </c>
       <c r="G181" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H181" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I181" s="6">
+      <c r="I181" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="B182" s="1" t="s">
         <v>763</v>
-      </c>
-      <c r="B182" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D182" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="E182" s="1" t="s">
         <v>764</v>
       </c>
-      <c r="E182" s="1" t="s">
+      <c r="F182" s="1" t="s">
         <v>765</v>
       </c>
-      <c r="F182" s="1" t="s">
-        <v>766</v>
-      </c>
       <c r="G182" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H182" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I182" s="6">
+      <c r="I182" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>768</v>
+        <v>171</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D183" s="1" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="E183" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="F183" s="1" t="s">
         <v>769</v>
       </c>
-      <c r="F183" s="1" t="s">
-        <v>770</v>
-      </c>
       <c r="G183" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H183" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I183" s="6">
+      <c r="I183" s="7">
         <v>46118.568367997686</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="B184" s="1" t="s">
         <v>771</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="C184" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D184" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="E184" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="F184" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="G184" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H184" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I184" s="7">
+        <v>46118.568367997686</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A185" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="B185" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="C184" s="1" t="s">
+      <c r="C185" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D184" s="1" t="s">
-        <v>772</v>
-      </c>
-      <c r="E184" s="1" t="s">
-        <v>773</v>
-      </c>
-      <c r="F184" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="G184" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H184" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I184" s="6">
-        <v>46118.568367997686</v>
+      <c r="D185" s="1" t="s">
+        <v>775</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="F185" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="G185" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H185" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I185" s="7">
+        <v>46118.568367997686</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A186" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D186" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="E186" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="F186" t="s">
+        <v>781</v>
+      </c>
+      <c r="G186" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H186" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I186" s="1"/>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="C187" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D187" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="E187" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="F187" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="G187" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H187" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I187" s="7">
+        <v>46119.801805555559</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A188" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D188" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="E188" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="F188" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="G188" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H188" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I188" s="7">
+        <v>46126.571747685186</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D189" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E189" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="F189" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="G189" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H189" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I189" s="7">
+        <v>46128.751099537039</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H184">
-    <sortCondition ref="D2:D184"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H185">
+    <sortCondition ref="D2:D185"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -8453,16 +8621,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21065E3C-A718-4C68-867F-24F90DCB0AB2}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="32" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -8473,7 +8641,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>775</v>
+        <v>794</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -8508,7 +8676,7 @@
         <v>383</v>
       </c>
       <c r="C2" t="s">
-        <v>776</v>
+        <v>384</v>
       </c>
       <c r="D2" t="s">
         <v>23</v>
@@ -8519,7 +8687,7 @@
       <c r="F2" t="s">
         <v>385</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" t="s">
         <v>386</v>
       </c>
       <c r="H2" t="s">
@@ -8529,48 +8697,13 @@
         <v>20</v>
       </c>
       <c r="J2" s="6">
-        <v>46119.568368055552</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="B3" t="s">
-        <v>485</v>
-      </c>
-      <c r="C3" t="s">
-        <v>531</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="6">
-        <v>46119.568368055552</v>
+        <v>46118.565717592595</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{3884E265-17D9-462D-BB6C-468724DBBD67}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8797,6 +8930,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="30aff7f6-e59e-4da9-89fc-ab8594e23593">
@@ -8805,15 +8947,6 @@
     <TaxCatchAll xmlns="4e599274-3222-4cb5-ba5a-ff9704aa99fe" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8836,6 +8969,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E255CF8B-FB3D-452B-BD35-7A8462448236}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D4D0E13-EB2A-4D5B-A887-D99E862CE6BA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -8844,12 +8985,4 @@
     <ds:schemaRef ds:uri="4e599274-3222-4cb5-ba5a-ff9704aa99fe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E255CF8B-FB3D-452B-BD35-7A8462448236}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>